<commit_message>
data: hourly update 2026-07-14 06:17Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 23:27</t>
+          <t>2026-07-14 02:17</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3292,32 +3292,32 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Portland Fire @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5426</v>
+        <v>0.6123</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-119</v>
+        <v>-158</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 61.2% (fair -158). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -3358,12 +3358,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -3373,17 +3373,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5499000000000001</v>
+        <v>0.5342</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-122</v>
+        <v>-115</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -3419,37 +3419,37 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Seattle Storm @ Chicago Sky</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +0.5</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.54</v>
+        <v>0.5678</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-117</v>
+        <v>-131</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 56.8% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -3482,9 +3482,339 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Washington Mystics @ Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Toronto Tempo +1.5</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>0.5542</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>-124</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>-104</v>
+      </c>
+      <c r="I8" s="13">
+        <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
+        <v/>
+      </c>
+      <c r="J8" s="16">
+        <f>IF($H$8="","",$F$8*IF($H$8&lt;0,-100/$H$8,$H$8/100)-(1-$F$8))</f>
+        <v/>
+      </c>
+      <c r="K8" s="17">
+        <f>IF($H$8="","",MAX(0,($F$8*IF($H$8&lt;0,-100/$H$8,$H$8/100)-(1-$F$8))/IF($H$8&lt;0,-100/$H$8,$H$8/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L8" s="18">
+        <f>IF($H$8="","",ROUND(MIN($K$8,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M8" s="12">
+        <f>IF($J$8="","",IF($J$8&lt;0,"Pass",IF($J$8&lt;'Settings'!$B$4,"Thin",IF($J$8&lt;0.06,"✅ Sharp band",IF($J$8&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N8" s="19" t="inlineStr">
+        <is>
+          <t>Model 55.4% (fair -124). Your call.</t>
+        </is>
+      </c>
+      <c r="O8" s="15" t="n"/>
+      <c r="P8" s="16">
+        <f>IF(OR($H$8="",$O$8=""),"",(1+IF($H$8&lt;0,-100/$H$8,$H$8/100))/(1+IF($O$8&lt;0,-100/$O$8,$O$8/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Washington Mystics @ Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Over 173.5</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>0.5165</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-107</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I9" s="13">
+        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
+        <v/>
+      </c>
+      <c r="K9" s="17">
+        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L9" s="18">
+        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M9" s="12">
+        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Model 51.6% (fair -107). Your call.</t>
+        </is>
+      </c>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="16">
+        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Portland Fire @ Connecticut Sun</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Connecticut Sun</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>0.5475</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-121</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>-104</v>
+      </c>
+      <c r="I10" s="13">
+        <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>IF($H$10="","",$F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))</f>
+        <v/>
+      </c>
+      <c r="K10" s="17">
+        <f>IF($H$10="","",MAX(0,($F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))/IF($H$10&lt;0,-100/$H$10,$H$10/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L10" s="18">
+        <f>IF($H$10="","",ROUND(MIN($K$10,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M10" s="12">
+        <f>IF($J$10="","",IF($J$10&lt;0,"Pass",IF($J$10&lt;'Settings'!$B$4,"Thin",IF($J$10&lt;0.06,"✅ Sharp band",IF($J$10&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.8% (fair -121). Your call.</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="16">
+        <f>IF(OR($H$10="",$O$10=""),"",(1+IF($H$10&lt;0,-100/$H$10,$H$10/100))/(1+IF($O$10&lt;0,-100/$O$10,$O$10/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Over 168.5</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>0.5417999999999999</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="I11" s="13">
+        <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>IF($H$11="","",$F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>IF($H$11="","",MAX(0,($F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))/IF($H$11&lt;0,-100/$H$11,$H$11/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L11" s="18">
+        <f>IF($H$11="","",ROUND(MIN($K$11,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M11" s="12">
+        <f>IF($J$11="","",IF($J$11&lt;0,"Pass",IF($J$11&lt;'Settings'!$B$4,"Thin",IF($J$11&lt;0.06,"✅ Sharp band",IF($J$11&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.2% (fair -118). Your call.</t>
+        </is>
+      </c>
+      <c r="O11" s="15" t="n"/>
+      <c r="P11" s="16">
+        <f>IF(OR($H$11="",$O$11=""),"",(1+IF($H$11&lt;0,-100/$H$11,$H$11/100))/(1+IF($O$11&lt;0,-100/$O$11,$O$11/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>Over 180.5</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>0.5339</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>-104</v>
+      </c>
+      <c r="I12" s="13">
+        <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
+        <v/>
+      </c>
+      <c r="J12" s="16">
+        <f>IF($H$12="","",$F$12*IF($H$12&lt;0,-100/$H$12,$H$12/100)-(1-$F$12))</f>
+        <v/>
+      </c>
+      <c r="K12" s="17">
+        <f>IF($H$12="","",MAX(0,($F$12*IF($H$12&lt;0,-100/$H$12,$H$12/100)-(1-$F$12))/IF($H$12&lt;0,-100/$H$12,$H$12/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L12" s="18">
+        <f>IF($H$12="","",ROUND(MIN($K$12,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M12" s="12">
+        <f>IF($J$12="","",IF($J$12&lt;0,"Pass",IF($J$12&lt;'Settings'!$B$4,"Thin",IF($J$12&lt;0.06,"✅ Sharp band",IF($J$12&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N12" s="19" t="inlineStr">
+        <is>
+          <t>Model 53.4% (fair -115). Your call.</t>
+        </is>
+      </c>
+      <c r="O12" s="15" t="n"/>
+      <c r="P12" s="16">
+        <f>IF(OR($H$12="",$O$12=""),"",(1+IF($H$12&lt;0,-100/$H$12,$H$12/100))/(1+IF($O$12&lt;0,-100/$O$12,$O$12/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J7">
+  <conditionalFormatting sqref="J5:J12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -3775,7 +4105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3919,13 +4249,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4500999999999999</v>
+        <v>0.4525</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -3949,7 +4279,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.0% (fair +122). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -3985,10 +4315,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5499000000000001</v>
+        <v>0.5475</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-122</v>
+        <v>-121</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-104</v>
@@ -4015,7 +4345,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -4047,17 +4377,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 168</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.7146628913991295</v>
+        <v>0.6123</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-250</v>
+        <v>-158</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -4081,7 +4411,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 71.5% (fair -250). Your call.</t>
+          <t>Model 61.2% (fair -158). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -4113,17 +4443,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 168</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.2653371086008705</v>
+        <v>0.3877</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>277</v>
+        <v>158</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -4147,7 +4477,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 26.5% (fair +277). Your call.</t>
+          <t>Model 38.8% (fair +158). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -4189,7 +4519,7 @@
         <v>103</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -4315,13 +4645,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4574</v>
+        <v>0.4658</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>102</v>
+        <v>-108</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -4345,7 +4675,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -4381,13 +4711,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5426</v>
+        <v>0.5342</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-119</v>
+        <v>-115</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -4411,7 +4741,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -4443,17 +4773,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 172.5</t>
+          <t>Over 173.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5661066863084717</v>
+        <v>0.5165</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-130</v>
+        <v>-107</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -4477,7 +4807,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -130). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -4509,17 +4839,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 172.5</t>
+          <t>Under 173.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4338933136915283</v>
+        <v>0.4835</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>130</v>
+        <v>107</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -4543,7 +4873,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +130). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -4575,17 +4905,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +0.5</t>
+          <t>Toronto Tempo +1.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.54</v>
+        <v>0.5542</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-117</v>
+        <v>-124</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-106</v>
+        <v>-104</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -4609,7 +4939,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 55.4% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -4641,14 +4971,14 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics -0.5</t>
+          <t>Washington Mystics -1.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.46</v>
+        <v>0.4458</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>104</v>
@@ -4675,7 +5005,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 44.6% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -4684,9 +5014,1197 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Seattle Storm</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>0.4071746000000001</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>146</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <v>156</v>
+      </c>
+      <c r="I17" s="13">
+        <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
+        <v/>
+      </c>
+      <c r="J17" s="16">
+        <f>IF($H$17="","",$F$17*IF($H$17&lt;0,-100/$H$17,$H$17/100)-(1-$F$17))</f>
+        <v/>
+      </c>
+      <c r="K17" s="17">
+        <f>IF($H$17="","",MAX(0,($F$17*IF($H$17&lt;0,-100/$H$17,$H$17/100)-(1-$F$17))/IF($H$17&lt;0,-100/$H$17,$H$17/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L17" s="18">
+        <f>IF($H$17="","",ROUND(MIN($K$17,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M17" s="12">
+        <f>IF($J$17="","",IF($J$17&lt;0,"Pass",IF($J$17&lt;'Settings'!$B$4,"Thin",IF($J$17&lt;0.06,"✅ Sharp band",IF($J$17&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N17" s="19" t="inlineStr">
+        <is>
+          <t>Model 40.7% (fair +146). Your call.</t>
+        </is>
+      </c>
+      <c r="O17" s="15" t="n"/>
+      <c r="P17" s="16">
+        <f>IF(OR($H$17="",$O$17=""),"",(1+IF($H$17&lt;0,-100/$H$17,$H$17/100))/(1+IF($O$17&lt;0,-100/$O$17,$O$17/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Chicago Sky</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.5928253999999999</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-146</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I18" s="13">
+        <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
+        <v/>
+      </c>
+      <c r="J18" s="16">
+        <f>IF($H$18="","",$F$18*IF($H$18&lt;0,-100/$H$18,$H$18/100)-(1-$F$18))</f>
+        <v/>
+      </c>
+      <c r="K18" s="17">
+        <f>IF($H$18="","",MAX(0,($F$18*IF($H$18&lt;0,-100/$H$18,$H$18/100)-(1-$F$18))/IF($H$18&lt;0,-100/$H$18,$H$18/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L18" s="18">
+        <f>IF($H$18="","",ROUND(MIN($K$18,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M18" s="12">
+        <f>IF($J$18="","",IF($J$18&lt;0,"Pass",IF($J$18&lt;'Settings'!$B$4,"Thin",IF($J$18&lt;0.06,"✅ Sharp band",IF($J$18&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N18" s="19" t="inlineStr">
+        <is>
+          <t>Model 59.3% (fair -146). Your call.</t>
+        </is>
+      </c>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="16">
+        <f>IF(OR($H$18="",$O$18=""),"",(1+IF($H$18&lt;0,-100/$H$18,$H$18/100))/(1+IF($O$18&lt;0,-100/$O$18,$O$18/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Over 170.5</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0.5678</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>-131</v>
+      </c>
+      <c r="H19" s="15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="I19" s="13">
+        <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>IF($H$19="","",$F$19*IF($H$19&lt;0,-100/$H$19,$H$19/100)-(1-$F$19))</f>
+        <v/>
+      </c>
+      <c r="K19" s="17">
+        <f>IF($H$19="","",MAX(0,($F$19*IF($H$19&lt;0,-100/$H$19,$H$19/100)-(1-$F$19))/IF($H$19&lt;0,-100/$H$19,$H$19/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L19" s="18">
+        <f>IF($H$19="","",ROUND(MIN($K$19,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M19" s="12">
+        <f>IF($J$19="","",IF($J$19&lt;0,"Pass",IF($J$19&lt;'Settings'!$B$4,"Thin",IF($J$19&lt;0.06,"✅ Sharp band",IF($J$19&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N19" s="19" t="inlineStr">
+        <is>
+          <t>Model 56.8% (fair -131). Your call.</t>
+        </is>
+      </c>
+      <c r="O19" s="15" t="n"/>
+      <c r="P19" s="16">
+        <f>IF(OR($H$19="",$O$19=""),"",(1+IF($H$19&lt;0,-100/$H$19,$H$19/100))/(1+IF($O$19&lt;0,-100/$O$19,$O$19/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>Under 170.5</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.4322</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>131</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v>-108</v>
+      </c>
+      <c r="I20" s="13">
+        <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
+        <v/>
+      </c>
+      <c r="J20" s="16">
+        <f>IF($H$20="","",$F$20*IF($H$20&lt;0,-100/$H$20,$H$20/100)-(1-$F$20))</f>
+        <v/>
+      </c>
+      <c r="K20" s="17">
+        <f>IF($H$20="","",MAX(0,($F$20*IF($H$20&lt;0,-100/$H$20,$H$20/100)-(1-$F$20))/IF($H$20&lt;0,-100/$H$20,$H$20/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L20" s="18">
+        <f>IF($H$20="","",ROUND(MIN($K$20,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M20" s="12">
+        <f>IF($J$20="","",IF($J$20&lt;0,"Pass",IF($J$20&lt;'Settings'!$B$4,"Thin",IF($J$20&lt;0.06,"✅ Sharp band",IF($J$20&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N20" s="19" t="inlineStr">
+        <is>
+          <t>Model 43.2% (fair +131). Your call.</t>
+        </is>
+      </c>
+      <c r="O20" s="15" t="n"/>
+      <c r="P20" s="16">
+        <f>IF(OR($H$20="",$O$20=""),"",(1+IF($H$20&lt;0,-100/$H$20,$H$20/100))/(1+IF($O$20&lt;0,-100/$O$20,$O$20/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Chicago Sky -3.5</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0.4948</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I21" s="13">
+        <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
+        <v/>
+      </c>
+      <c r="J21" s="16">
+        <f>IF($H$21="","",$F$21*IF($H$21&lt;0,-100/$H$21,$H$21/100)-(1-$F$21))</f>
+        <v/>
+      </c>
+      <c r="K21" s="17">
+        <f>IF($H$21="","",MAX(0,($F$21*IF($H$21&lt;0,-100/$H$21,$H$21/100)-(1-$F$21))/IF($H$21&lt;0,-100/$H$21,$H$21/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L21" s="18">
+        <f>IF($H$21="","",ROUND(MIN($K$21,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M21" s="12">
+        <f>IF($J$21="","",IF($J$21&lt;0,"Pass",IF($J$21&lt;'Settings'!$B$4,"Thin",IF($J$21&lt;0.06,"✅ Sharp band",IF($J$21&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N21" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.5% (fair +102). Your call.</t>
+        </is>
+      </c>
+      <c r="O21" s="15" t="n"/>
+      <c r="P21" s="16">
+        <f>IF(OR($H$21="",$O$21=""),"",(1+IF($H$21&lt;0,-100/$H$21,$H$21/100))/(1+IF($O$21&lt;0,-100/$O$21,$O$21/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Storm +3.5</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.5052</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>-102</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v>-106</v>
+      </c>
+      <c r="I22" s="13">
+        <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
+        <v/>
+      </c>
+      <c r="J22" s="16">
+        <f>IF($H$22="","",$F$22*IF($H$22&lt;0,-100/$H$22,$H$22/100)-(1-$F$22))</f>
+        <v/>
+      </c>
+      <c r="K22" s="17">
+        <f>IF($H$22="","",MAX(0,($F$22*IF($H$22&lt;0,-100/$H$22,$H$22/100)-(1-$F$22))/IF($H$22&lt;0,-100/$H$22,$H$22/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L22" s="18">
+        <f>IF($H$22="","",ROUND(MIN($K$22,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M22" s="12">
+        <f>IF($J$22="","",IF($J$22&lt;0,"Pass",IF($J$22&lt;'Settings'!$B$4,"Thin",IF($J$22&lt;0.06,"✅ Sharp band",IF($J$22&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N22" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.5% (fair -102). Your call.</t>
+        </is>
+      </c>
+      <c r="O22" s="15" t="n"/>
+      <c r="P22" s="16">
+        <f>IF(OR($H$22="",$O$22=""),"",(1+IF($H$22&lt;0,-100/$H$22,$H$22/100))/(1+IF($O$22&lt;0,-100/$O$22,$O$22/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>0.07955000000000001</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>1157</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>570</v>
+      </c>
+      <c r="I23" s="13">
+        <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
+        <v/>
+      </c>
+      <c r="J23" s="16">
+        <f>IF($H$23="","",$F$23*IF($H$23&lt;0,-100/$H$23,$H$23/100)-(1-$F$23))</f>
+        <v/>
+      </c>
+      <c r="K23" s="17">
+        <f>IF($H$23="","",MAX(0,($F$23*IF($H$23&lt;0,-100/$H$23,$H$23/100)-(1-$F$23))/IF($H$23&lt;0,-100/$H$23,$H$23/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L23" s="18">
+        <f>IF($H$23="","",ROUND(MIN($K$23,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M23" s="12">
+        <f>IF($J$23="","",IF($J$23&lt;0,"Pass",IF($J$23&lt;'Settings'!$B$4,"Thin",IF($J$23&lt;0.06,"✅ Sharp band",IF($J$23&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N23" s="19" t="inlineStr">
+        <is>
+          <t>Model 8.0% (fair +1157). Your call.</t>
+        </is>
+      </c>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="16">
+        <f>IF(OR($H$23="",$O$23=""),"",(1+IF($H$23&lt;0,-100/$H$23,$H$23/100))/(1+IF($O$23&lt;0,-100/$O$23,$O$23/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.92045</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-1157</v>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I24" s="13">
+        <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
+        <v/>
+      </c>
+      <c r="J24" s="16">
+        <f>IF($H$24="","",$F$24*IF($H$24&lt;0,-100/$H$24,$H$24/100)-(1-$F$24))</f>
+        <v/>
+      </c>
+      <c r="K24" s="17">
+        <f>IF($H$24="","",MAX(0,($F$24*IF($H$24&lt;0,-100/$H$24,$H$24/100)-(1-$F$24))/IF($H$24&lt;0,-100/$H$24,$H$24/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L24" s="18">
+        <f>IF($H$24="","",ROUND(MIN($K$24,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M24" s="12">
+        <f>IF($J$24="","",IF($J$24&lt;0,"Pass",IF($J$24&lt;'Settings'!$B$4,"Thin",IF($J$24&lt;0.06,"✅ Sharp band",IF($J$24&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N24" s="19" t="inlineStr">
+        <is>
+          <t>Model 92.0% (fair -1157). Your call.</t>
+        </is>
+      </c>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="16">
+        <f>IF(OR($H$24="",$O$24=""),"",(1+IF($H$24&lt;0,-100/$H$24,$H$24/100))/(1+IF($O$24&lt;0,-100/$O$24,$O$24/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Over 180.5</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>0.5339</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v>-104</v>
+      </c>
+      <c r="I25" s="13">
+        <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
+        <v/>
+      </c>
+      <c r="J25" s="16">
+        <f>IF($H$25="","",$F$25*IF($H$25&lt;0,-100/$H$25,$H$25/100)-(1-$F$25))</f>
+        <v/>
+      </c>
+      <c r="K25" s="17">
+        <f>IF($H$25="","",MAX(0,($F$25*IF($H$25&lt;0,-100/$H$25,$H$25/100)-(1-$F$25))/IF($H$25&lt;0,-100/$H$25,$H$25/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>IF($H$25="","",ROUND(MIN($K$25,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M25" s="12">
+        <f>IF($J$25="","",IF($J$25&lt;0,"Pass",IF($J$25&lt;'Settings'!$B$4,"Thin",IF($J$25&lt;0.06,"✅ Sharp band",IF($J$25&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N25" s="19" t="inlineStr">
+        <is>
+          <t>Model 53.4% (fair -115). Your call.</t>
+        </is>
+      </c>
+      <c r="O25" s="15" t="n"/>
+      <c r="P25" s="16">
+        <f>IF(OR($H$25="",$O$25=""),"",(1+IF($H$25&lt;0,-100/$H$25,$H$25/100))/(1+IF($O$25&lt;0,-100/$O$25,$O$25/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Under 180.5</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.4661</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>115</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="I26" s="13">
+        <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
+        <v/>
+      </c>
+      <c r="J26" s="16">
+        <f>IF($H$26="","",$F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))</f>
+        <v/>
+      </c>
+      <c r="K26" s="17">
+        <f>IF($H$26="","",MAX(0,($F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))/IF($H$26&lt;0,-100/$H$26,$H$26/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
+        <f>IF($H$26="","",ROUND(MIN($K$26,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M26" s="12">
+        <f>IF($J$26="","",IF($J$26&lt;0,"Pass",IF($J$26&lt;'Settings'!$B$4,"Thin",IF($J$26&lt;0.06,"✅ Sharp band",IF($J$26&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>Model 46.6% (fair +115). Your call.</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="16">
+        <f>IF(OR($H$26="",$O$26=""),"",(1+IF($H$26&lt;0,-100/$H$26,$H$26/100))/(1+IF($O$26&lt;0,-100/$O$26,$O$26/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx -12.5</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0.4906</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>104</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v>-108</v>
+      </c>
+      <c r="I27" s="13">
+        <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
+        <v/>
+      </c>
+      <c r="J27" s="16">
+        <f>IF($H$27="","",$F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))</f>
+        <v/>
+      </c>
+      <c r="K27" s="17">
+        <f>IF($H$27="","",MAX(0,($F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))/IF($H$27&lt;0,-100/$H$27,$H$27/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
+        <f>IF($H$27="","",ROUND(MIN($K$27,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M27" s="12">
+        <f>IF($J$27="","",IF($J$27&lt;0,"Pass",IF($J$27&lt;'Settings'!$B$4,"Thin",IF($J$27&lt;0.06,"✅ Sharp band",IF($J$27&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N27" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.1% (fair +104). Your call.</t>
+        </is>
+      </c>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="16">
+        <f>IF(OR($H$27="",$O$27=""),"",(1+IF($H$27&lt;0,-100/$H$27,$H$27/100))/(1+IF($O$27&lt;0,-100/$O$27,$O$27/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks +12.5</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.5094000000000001</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>-104</v>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v>-106</v>
+      </c>
+      <c r="I28" s="13">
+        <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
+        <v/>
+      </c>
+      <c r="J28" s="16">
+        <f>IF($H$28="","",$F$28*IF($H$28&lt;0,-100/$H$28,$H$28/100)-(1-$F$28))</f>
+        <v/>
+      </c>
+      <c r="K28" s="17">
+        <f>IF($H$28="","",MAX(0,($F$28*IF($H$28&lt;0,-100/$H$28,$H$28/100)-(1-$F$28))/IF($H$28&lt;0,-100/$H$28,$H$28/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
+        <f>IF($H$28="","",ROUND(MIN($K$28,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M28" s="12">
+        <f>IF($J$28="","",IF($J$28&lt;0,"Pass",IF($J$28&lt;'Settings'!$B$4,"Thin",IF($J$28&lt;0.06,"✅ Sharp band",IF($J$28&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N28" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.9% (fair -104). Your call.</t>
+        </is>
+      </c>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="16">
+        <f>IF(OR($H$28="",$O$28=""),"",(1+IF($H$28&lt;0,-100/$H$28,$H$28/100))/(1+IF($O$28&lt;0,-100/$O$28,$O$28/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0.445452</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>124</v>
+      </c>
+      <c r="H29" s="15" t="n">
+        <v>122</v>
+      </c>
+      <c r="I29" s="13">
+        <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
+        <v/>
+      </c>
+      <c r="J29" s="16">
+        <f>IF($H$29="","",$F$29*IF($H$29&lt;0,-100/$H$29,$H$29/100)-(1-$F$29))</f>
+        <v/>
+      </c>
+      <c r="K29" s="17">
+        <f>IF($H$29="","",MAX(0,($F$29*IF($H$29&lt;0,-100/$H$29,$H$29/100)-(1-$F$29))/IF($H$29&lt;0,-100/$H$29,$H$29/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L29" s="18">
+        <f>IF($H$29="","",ROUND(MIN($K$29,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M29" s="12">
+        <f>IF($J$29="","",IF($J$29&lt;0,"Pass",IF($J$29&lt;'Settings'!$B$4,"Thin",IF($J$29&lt;0.06,"✅ Sharp band",IF($J$29&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N29" s="19" t="inlineStr">
+        <is>
+          <t>Model 44.5% (fair +124). Your call.</t>
+        </is>
+      </c>
+      <c r="O29" s="15" t="n"/>
+      <c r="P29" s="16">
+        <f>IF(OR($H$29="",$O$29=""),"",(1+IF($H$29&lt;0,-100/$H$29,$H$29/100))/(1+IF($O$29&lt;0,-100/$O$29,$O$29/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.554548</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>-124</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <v>-108</v>
+      </c>
+      <c r="I30" s="13">
+        <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
+        <v/>
+      </c>
+      <c r="J30" s="16">
+        <f>IF($H$30="","",$F$30*IF($H$30&lt;0,-100/$H$30,$H$30/100)-(1-$F$30))</f>
+        <v/>
+      </c>
+      <c r="K30" s="17">
+        <f>IF($H$30="","",MAX(0,($F$30*IF($H$30&lt;0,-100/$H$30,$H$30/100)-(1-$F$30))/IF($H$30&lt;0,-100/$H$30,$H$30/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L30" s="18">
+        <f>IF($H$30="","",ROUND(MIN($K$30,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M30" s="12">
+        <f>IF($J$30="","",IF($J$30&lt;0,"Pass",IF($J$30&lt;'Settings'!$B$4,"Thin",IF($J$30&lt;0.06,"✅ Sharp band",IF($J$30&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N30" s="19" t="inlineStr">
+        <is>
+          <t>Model 55.5% (fair -124). Your call.</t>
+        </is>
+      </c>
+      <c r="O30" s="15" t="n"/>
+      <c r="P30" s="16">
+        <f>IF(OR($H$30="",$O$30=""),"",(1+IF($H$30&lt;0,-100/$H$30,$H$30/100))/(1+IF($O$30&lt;0,-100/$O$30,$O$30/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Over 168.5</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="n">
+        <v>0.5417999999999999</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H31" s="15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="I31" s="13">
+        <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
+        <v/>
+      </c>
+      <c r="J31" s="16">
+        <f>IF($H$31="","",$F$31*IF($H$31&lt;0,-100/$H$31,$H$31/100)-(1-$F$31))</f>
+        <v/>
+      </c>
+      <c r="K31" s="17">
+        <f>IF($H$31="","",MAX(0,($F$31*IF($H$31&lt;0,-100/$H$31,$H$31/100)-(1-$F$31))/IF($H$31&lt;0,-100/$H$31,$H$31/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L31" s="18">
+        <f>IF($H$31="","",ROUND(MIN($K$31,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M31" s="12">
+        <f>IF($J$31="","",IF($J$31&lt;0,"Pass",IF($J$31&lt;'Settings'!$B$4,"Thin",IF($J$31&lt;0.06,"✅ Sharp band",IF($J$31&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N31" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.2% (fair -118). Your call.</t>
+        </is>
+      </c>
+      <c r="O31" s="15" t="n"/>
+      <c r="P31" s="16">
+        <f>IF(OR($H$31="",$O$31=""),"",(1+IF($H$31&lt;0,-100/$H$31,$H$31/100))/(1+IF($O$31&lt;0,-100/$O$31,$O$31/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>Under 168.5</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>0.4582000000000001</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>118</v>
+      </c>
+      <c r="H32" s="15" t="n">
+        <v>113</v>
+      </c>
+      <c r="I32" s="13">
+        <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
+        <v/>
+      </c>
+      <c r="J32" s="16">
+        <f>IF($H$32="","",$F$32*IF($H$32&lt;0,-100/$H$32,$H$32/100)-(1-$F$32))</f>
+        <v/>
+      </c>
+      <c r="K32" s="17">
+        <f>IF($H$32="","",MAX(0,($F$32*IF($H$32&lt;0,-100/$H$32,$H$32/100)-(1-$F$32))/IF($H$32&lt;0,-100/$H$32,$H$32/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L32" s="18">
+        <f>IF($H$32="","",ROUND(MIN($K$32,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M32" s="12">
+        <f>IF($J$32="","",IF($J$32&lt;0,"Pass",IF($J$32&lt;'Settings'!$B$4,"Thin",IF($J$32&lt;0.06,"✅ Sharp band",IF($J$32&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N32" s="19" t="inlineStr">
+        <is>
+          <t>Model 45.8% (fair +118). Your call.</t>
+        </is>
+      </c>
+      <c r="O32" s="15" t="n"/>
+      <c r="P32" s="16">
+        <f>IF(OR($H$32="",$O$32=""),"",(1+IF($H$32&lt;0,-100/$H$32,$H$32/100))/(1+IF($O$32&lt;0,-100/$O$32,$O$32/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Indiana Fever -1.5</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>103</v>
+      </c>
+      <c r="H33" s="15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="I33" s="13">
+        <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
+        <v/>
+      </c>
+      <c r="J33" s="16">
+        <f>IF($H$33="","",$F$33*IF($H$33&lt;0,-100/$H$33,$H$33/100)-(1-$F$33))</f>
+        <v/>
+      </c>
+      <c r="K33" s="17">
+        <f>IF($H$33="","",MAX(0,($F$33*IF($H$33&lt;0,-100/$H$33,$H$33/100)-(1-$F$33))/IF($H$33&lt;0,-100/$H$33,$H$33/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L33" s="18">
+        <f>IF($H$33="","",ROUND(MIN($K$33,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M33" s="12">
+        <f>IF($J$33="","",IF($J$33&lt;0,"Pass",IF($J$33&lt;'Settings'!$B$4,"Thin",IF($J$33&lt;0.06,"✅ Sharp band",IF($J$33&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N33" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.3% (fair +103). Your call.</t>
+        </is>
+      </c>
+      <c r="O33" s="15" t="n"/>
+      <c r="P33" s="16">
+        <f>IF(OR($H$33="",$O$33=""),"",(1+IF($H$33&lt;0,-100/$H$33,$H$33/100))/(1+IF($O$33&lt;0,-100/$O$33,$O$33/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D34" s="20" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E34" s="20" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries +1.5</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0.5074000000000001</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>-103</v>
+      </c>
+      <c r="H34" s="15" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I34" s="13">
+        <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
+        <v/>
+      </c>
+      <c r="J34" s="16">
+        <f>IF($H$34="","",$F$34*IF($H$34&lt;0,-100/$H$34,$H$34/100)-(1-$F$34))</f>
+        <v/>
+      </c>
+      <c r="K34" s="17">
+        <f>IF($H$34="","",MAX(0,($F$34*IF($H$34&lt;0,-100/$H$34,$H$34/100)-(1-$F$34))/IF($H$34&lt;0,-100/$H$34,$H$34/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L34" s="18">
+        <f>IF($H$34="","",ROUND(MIN($K$34,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M34" s="12">
+        <f>IF($J$34="","",IF($J$34&lt;0,"Pass",IF($J$34&lt;'Settings'!$B$4,"Thin",IF($J$34&lt;0.06,"✅ Sharp band",IF($J$34&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N34" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.7% (fair -103). Your call.</t>
+        </is>
+      </c>
+      <c r="O34" s="15" t="n"/>
+      <c r="P34" s="16">
+        <f>IF(OR($H$34="",$O$34=""),"",(1+IF($H$34&lt;0,-100/$H$34,$H$34/100))/(1+IF($O$34&lt;0,-100/$O$34,$O$34/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J16">
+  <conditionalFormatting sqref="J5:J34">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 14:57Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 02:17</t>
+          <t>2026-07-14 10:57</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3292,32 +3292,32 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6123</v>
+        <v>0.529</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-158</v>
+        <v>-112</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -3353,37 +3353,37 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Seattle Storm @ Chicago Sky</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5342</v>
+        <v>0.5778</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-115</v>
+        <v>-137</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>108</v>
+        <v>-110</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -3419,17 +3419,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Chicago Sky</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -3439,17 +3439,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Over 173.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5678</v>
+        <v>0.5165</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-131</v>
+        <v>-107</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-105</v>
+        <v>108</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -131). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -3485,37 +3485,37 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Golden State Valkyries @ Indiana Fever</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo +1.5</t>
+          <t>Over 168.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5542</v>
+        <v>0.5334</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-124</v>
+        <v>-114</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 55.4% (fair -124). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -3551,17 +3551,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -3571,17 +3571,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 180.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5165</v>
+        <v>0.5441</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-107</v>
+        <v>-119</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>-108</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -3617,17 +3617,17 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Golden State Valkyries @ Indiana Fever</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -3637,17 +3637,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5475</v>
+        <v>0.5448</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-121</v>
+        <v>-120</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-104</v>
+        <v>-113</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -3680,141 +3680,9 @@
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Over 168.5</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="n">
-        <v>0.5417999999999999</v>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>-118</v>
-      </c>
-      <c r="H11" s="15" t="n">
-        <v>-105</v>
-      </c>
-      <c r="I11" s="13">
-        <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
-        <v/>
-      </c>
-      <c r="J11" s="16">
-        <f>IF($H$11="","",$F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="17">
-        <f>IF($H$11="","",MAX(0,($F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))/IF($H$11&lt;0,-100/$H$11,$H$11/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L11" s="18">
-        <f>IF($H$11="","",ROUND(MIN($K$11,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M11" s="12">
-        <f>IF($J$11="","",IF($J$11&lt;0,"Pass",IF($J$11&lt;'Settings'!$B$4,"Thin",IF($J$11&lt;0.06,"✅ Sharp band",IF($J$11&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N11" s="19" t="inlineStr">
-        <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
-        </is>
-      </c>
-      <c r="O11" s="15" t="n"/>
-      <c r="P11" s="16">
-        <f>IF(OR($H$11="",$O$11=""),"",(1+IF($H$11&lt;0,-100/$H$11,$H$11/100))/(1+IF($O$11&lt;0,-100/$O$11,$O$11/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks @ Minnesota Lynx</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>Over 180.5</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="n">
-        <v>0.5339</v>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>-115</v>
-      </c>
-      <c r="H12" s="15" t="n">
-        <v>-104</v>
-      </c>
-      <c r="I12" s="13">
-        <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
-        <v/>
-      </c>
-      <c r="J12" s="16">
-        <f>IF($H$12="","",$F$12*IF($H$12&lt;0,-100/$H$12,$H$12/100)-(1-$F$12))</f>
-        <v/>
-      </c>
-      <c r="K12" s="17">
-        <f>IF($H$12="","",MAX(0,($F$12*IF($H$12&lt;0,-100/$H$12,$H$12/100)-(1-$F$12))/IF($H$12&lt;0,-100/$H$12,$H$12/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L12" s="18">
-        <f>IF($H$12="","",ROUND(MIN($K$12,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M12" s="12">
-        <f>IF($J$12="","",IF($J$12&lt;0,"Pass",IF($J$12&lt;'Settings'!$B$4,"Thin",IF($J$12&lt;0.06,"✅ Sharp band",IF($J$12&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N12" s="19" t="inlineStr">
-        <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
-        </is>
-      </c>
-      <c r="O12" s="15" t="n"/>
-      <c r="P12" s="16">
-        <f>IF(OR($H$12="",$O$12=""),"",(1+IF($H$12&lt;0,-100/$H$12,$H$12/100))/(1+IF($O$12&lt;0,-100/$O$12,$O$12/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J12">
+  <conditionalFormatting sqref="J5:J10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -3980,10 +3848,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5006</v>
+        <v>0.4992</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="H5" s="15" t="n"/>
       <c r="I5" s="13">
@@ -4008,7 +3876,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -4044,10 +3912,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.4995</v>
+        <v>0.5008</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>100</v>
+        <v>-100</v>
       </c>
       <c r="H6" s="15" t="n"/>
       <c r="I6" s="13">
@@ -4072,7 +3940,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair +100). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -4249,13 +4117,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4525</v>
+        <v>0.41237</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -4279,7 +4147,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 41.2% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -4315,13 +4183,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5475</v>
+        <v>0.58763</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-121</v>
+        <v>-143</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-104</v>
+        <v>-110</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -4345,7 +4213,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 58.8% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -4377,17 +4245,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 168</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6123</v>
+        <v>0.7146628913991295</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-158</v>
+        <v>-250</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -4411,7 +4279,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 71.5% (fair -250). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -4443,17 +4311,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 167.5</t>
+          <t>Under 168</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3877</v>
+        <v>0.2653371086008705</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>158</v>
+        <v>277</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -4477,7 +4345,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 26.5% (fair +277). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -4509,17 +4377,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun -1.5</t>
+          <t>Connecticut Sun -3.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4930895344612759</v>
+        <v>0.4306171567084904</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -4543,7 +4411,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 43.1% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -4575,17 +4443,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire +1.5</t>
+          <t>Portland Fire +3.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5069104655387241</v>
+        <v>0.5693828432915096</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-103</v>
+        <v>-132</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -4609,7 +4477,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 56.9% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -4645,13 +4513,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4658</v>
+        <v>0.471</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -4675,7 +4543,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 47.1% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -4711,13 +4579,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5342</v>
+        <v>0.529</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-115</v>
+        <v>-112</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -4741,7 +4609,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -4905,17 +4773,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +1.5</t>
+          <t>Toronto Tempo +0.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5542</v>
+        <v>0.5678354899577411</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-124</v>
+        <v>-131</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -4939,7 +4807,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 55.4% (fair -124). Your call.</t>
+          <t>Model 56.8% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -4971,17 +4839,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics -1.5</t>
+          <t>Washington Mystics -0.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4458</v>
+        <v>0.4321645100422589</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -5005,7 +4873,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 44.6% (fair +124). Your call.</t>
+          <t>Model 43.2% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -5047,7 +4915,7 @@
         <v>146</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -5113,7 +4981,7 @@
         <v>-146</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -5173,13 +5041,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5678</v>
+        <v>0.5778</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-131</v>
+        <v>-137</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5203,7 +5071,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -131). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -5239,13 +5107,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4322</v>
+        <v>0.4222</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-108</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -5269,7 +5137,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 43.2% (fair +131). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -5305,13 +5173,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4948</v>
+        <v>0.4926</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-110</v>
+        <v>-104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -5335,7 +5203,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -5371,13 +5239,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5052</v>
+        <v>0.5074000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-106</v>
+        <v>-104</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -5401,7 +5269,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -5443,7 +5311,7 @@
         <v>1157</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>570</v>
+        <v>614</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -5509,7 +5377,7 @@
         <v>-1157</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -5569,13 +5437,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5339</v>
+        <v>0.5441</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-115</v>
+        <v>-119</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -5599,7 +5467,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -5635,13 +5503,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4661</v>
+        <v>0.4559</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-105</v>
+        <v>108</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -5665,7 +5533,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -5701,13 +5569,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4906</v>
+        <v>0.4889</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -5731,7 +5599,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 48.9% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -5767,13 +5635,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5094000000000001</v>
+        <v>0.5111</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -5797,7 +5665,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 51.1% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -5833,13 +5701,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.445452</v>
+        <v>0.4552</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -5863,7 +5731,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +124). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -5899,13 +5767,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.554548</v>
+        <v>0.5448</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-124</v>
+        <v>-120</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-108</v>
+        <v>-113</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -5929,7 +5797,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -124). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -5965,13 +5833,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5417999999999999</v>
+        <v>0.5334</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-118</v>
+        <v>-114</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -5995,7 +5863,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -6031,13 +5899,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4582000000000001</v>
+        <v>0.4666</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -6061,7 +5929,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -6097,13 +5965,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.4926</v>
+        <v>0.4921</v>
       </c>
       <c r="G33" s="14" t="n">
         <v>103</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -6127,7 +5995,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -6163,7 +6031,7 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5074000000000001</v>
+        <v>0.5079</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>-103</v>
@@ -6193,7 +6061,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 15:48Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 10:57</t>
+          <t>2026-07-14 11:48</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3287,37 +3287,37 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Seattle Storm @ Chicago Sky</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.529</v>
+        <v>0.5768</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-112</v>
+        <v>-136</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>115</v>
+        <v>-104</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -3353,37 +3353,37 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Chicago Sky</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5778</v>
+        <v>0.5301</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-137</v>
+        <v>-113</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-110</v>
+        <v>113</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -3419,17 +3419,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -3439,17 +3439,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 180.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5165</v>
+        <v>0.5441</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-107</v>
+        <v>-119</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>-108</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -3509,13 +3509,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5334</v>
+        <v>0.5417</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-114</v>
+        <v>-118</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -3556,32 +3556,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+          <t>Golden State Valkyries @ Indiana Fever</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 180.5</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5441</v>
+        <v>0.5425</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>-119</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>-108</v>
+        <v>-113</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 54.2% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -3614,75 +3614,9 @@
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Indiana Fever</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>0.5448</v>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>-120</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <v>-113</v>
-      </c>
-      <c r="I10" s="13">
-        <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
-        <v/>
-      </c>
-      <c r="J10" s="16">
-        <f>IF($H$10="","",$F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="17">
-        <f>IF($H$10="","",MAX(0,($F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))/IF($H$10&lt;0,-100/$H$10,$H$10/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L10" s="18">
-        <f>IF($H$10="","",ROUND(MIN($K$10,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M10" s="12">
-        <f>IF($J$10="","",IF($J$10&lt;0,"Pass",IF($J$10&lt;'Settings'!$B$4,"Thin",IF($J$10&lt;0.06,"✅ Sharp band",IF($J$10&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N10" s="19" t="inlineStr">
-        <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
-        </is>
-      </c>
-      <c r="O10" s="15" t="n"/>
-      <c r="P10" s="16">
-        <f>IF(OR($H$10="",$O$10=""),"",(1+IF($H$10&lt;0,-100/$H$10,$H$10/100))/(1+IF($O$10&lt;0,-100/$O$10,$O$10/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J10">
+  <conditionalFormatting sqref="J5:J9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -4123,7 +4057,7 @@
         <v>143</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -4245,17 +4179,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 168</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.7146628913991295</v>
+        <v>0.7245695517138792</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-250</v>
+        <v>-263</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -4279,7 +4213,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 71.5% (fair -250). Your call.</t>
+          <t>Model 72.5% (fair -263). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -4311,17 +4245,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 168</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.2653371086008705</v>
+        <v>0.2754304482861208</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -4345,7 +4279,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 26.5% (fair +277). Your call.</t>
+          <t>Model 27.5% (fair +263). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -4453,7 +4387,7 @@
         <v>-132</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -4513,10 +4447,10 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.471</v>
+        <v>0.4699</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>-110</v>
@@ -4543,7 +4477,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -4579,13 +4513,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.529</v>
+        <v>0.5301</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-112</v>
+        <v>-113</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -4609,7 +4543,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -4645,13 +4579,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5165</v>
+        <v>0.5428621668460131</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-107</v>
+        <v>-119</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -4675,7 +4609,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -4711,13 +4645,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4835</v>
+        <v>0.4571378331539869</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>-103</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -4741,7 +4675,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -5041,13 +4975,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5778</v>
+        <v>0.5768</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-137</v>
+        <v>-136</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-110</v>
+        <v>-104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5071,7 +5005,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -5107,13 +5041,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4222</v>
+        <v>0.4232</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -5137,7 +5071,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.2% (fair +137). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -5173,10 +5107,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4926</v>
+        <v>0.495</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>-104</v>
@@ -5203,7 +5137,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -5239,13 +5173,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5074000000000001</v>
+        <v>0.505</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-103</v>
+        <v>-102</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -5269,7 +5203,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -5569,13 +5503,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4889</v>
+        <v>0.4865</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -5599,7 +5533,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +105). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -5635,10 +5569,10 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5111</v>
+        <v>0.5135000000000001</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>-105</v>
@@ -5665,7 +5599,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 51.1% (fair -105). Your call.</t>
+          <t>Model 51.4% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -5701,13 +5635,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4552</v>
+        <v>0.4575</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -5731,7 +5665,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 45.5% (fair +120). Your call.</t>
+          <t>Model 45.8% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -5767,10 +5701,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5448</v>
+        <v>0.5425</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-120</v>
+        <v>-119</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-113</v>
@@ -5797,7 +5731,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 54.2% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -5833,13 +5767,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5334</v>
+        <v>0.5417</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-114</v>
+        <v>-118</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -5863,7 +5797,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -5899,13 +5833,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4666</v>
+        <v>0.4583</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -5929,7 +5863,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -5965,13 +5899,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.4921</v>
+        <v>0.4883</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -5995,7 +5929,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 48.8% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -6031,13 +5965,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5079</v>
+        <v>0.5117</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-103</v>
+        <v>-105</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -6061,7 +5995,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 16:11Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 11:48</t>
+          <t>2026-07-14 12:11</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3287,37 +3287,37 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Chicago Sky</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5768</v>
+        <v>0.5286</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-136</v>
+        <v>-112</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-104</v>
+        <v>113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -3368,22 +3368,22 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Toronto Tempo +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5301</v>
+        <v>0.5493</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-113</v>
+        <v>-122</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -3424,12 +3424,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+          <t>Golden State Valkyries @ Indiana Fever</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -3439,17 +3439,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 180.5</t>
+          <t>Over 168.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5441</v>
+        <v>0.5359</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-119</v>
+        <v>-115</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -3490,12 +3490,12 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -3505,17 +3505,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>Over 180.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5417</v>
+        <v>0.5441</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-118</v>
+        <v>-119</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -3548,75 +3548,9 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Indiana Fever</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>0.5425</v>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>-119</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>-113</v>
-      </c>
-      <c r="I9" s="13">
-        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="16">
-        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="17">
-        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L9" s="18">
-        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M9" s="12">
-        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N9" s="19" t="inlineStr">
-        <is>
-          <t>Model 54.2% (fair -119). Your call.</t>
-        </is>
-      </c>
-      <c r="O9" s="15" t="n"/>
-      <c r="P9" s="16">
-        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J9">
+  <conditionalFormatting sqref="J5:J8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -4447,13 +4381,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4699</v>
+        <v>0.4714</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-110</v>
+        <v>-113</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -4477,7 +4411,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 47.1% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -4513,10 +4447,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5301</v>
+        <v>0.5286</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-113</v>
+        <v>-112</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>113</v>
@@ -4543,7 +4477,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -4651,7 +4585,7 @@
         <v>119</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-103</v>
+        <v>-102</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -4707,17 +4641,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +0.5</t>
+          <t>Toronto Tempo +1.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5678354899577411</v>
+        <v>0.5493</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-131</v>
+        <v>-122</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -4741,7 +4675,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -131). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -4773,17 +4707,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics -0.5</t>
+          <t>Washington Mystics -1.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4321645100422589</v>
+        <v>0.4507</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -4807,7 +4741,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 43.2% (fair +131). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -4971,17 +4905,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Over 172.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5768</v>
+        <v>0.5941506978584125</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-136</v>
+        <v>-146</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5005,7 +4939,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 59.4% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -5037,14 +4971,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 170.5</t>
+          <t>Under 172.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4232</v>
+        <v>0.4058493021415875</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>108</v>
@@ -5071,7 +5005,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 40.6% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -5503,13 +5437,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4865</v>
+        <v>0.4895</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -5533,7 +5467,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 48.6% (fair +106). Your call.</t>
+          <t>Model 48.9% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -5569,13 +5503,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5135000000000001</v>
+        <v>0.5105</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-106</v>
+        <v>-104</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -5599,7 +5533,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 51.4% (fair -106). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -5635,7 +5569,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4575</v>
+        <v>0.4564</v>
       </c>
       <c r="G29" s="14" t="n">
         <v>119</v>
@@ -5665,7 +5599,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +119). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -5701,13 +5635,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5425</v>
+        <v>0.5436</v>
       </c>
       <c r="G30" s="14" t="n">
         <v>-119</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -5731,7 +5665,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -119). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -5767,13 +5701,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5417</v>
+        <v>0.5359</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-118</v>
+        <v>-115</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -5797,7 +5731,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -5833,10 +5767,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4583</v>
+        <v>0.4641</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>108</v>
@@ -5863,7 +5797,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 46.4% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -5899,13 +5833,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.4883</v>
+        <v>0.4907</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -5929,7 +5863,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -5965,10 +5899,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5117</v>
+        <v>0.5093</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>-108</v>
@@ -5995,7 +5929,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 19:28Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="11668125"/>
+    <ext cx="10125075" cy="12192000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 14:08</t>
+          <t>2026-07-14 15:27</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5264</v>
+        <v>0.5286</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-111</v>
+        <v>-112</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5518</v>
+        <v>0.545</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-123</v>
+        <v>-120</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1377,32 +1377,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Los Angeles Sparks +12.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.508</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-120</v>
+        <v>-103</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>-115</v>
+        <v>104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.6% (fair -120). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -1435,9 +1435,141 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Under 183.5</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>0.4957</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I10" s="13">
+        <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>IF($H$10="","",$F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))</f>
+        <v/>
+      </c>
+      <c r="K10" s="17">
+        <f>IF($H$10="","",MAX(0,($F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))/IF($H$10&lt;0,-100/$H$10,$H$10/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L10" s="18">
+        <f>IF($H$10="","",ROUND(MIN($K$10,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M10" s="12">
+        <f>IF($J$10="","",IF($J$10&lt;0,"Pass",IF($J$10&lt;'Settings'!$B$4,"Thin",IF($J$10&lt;0.06,"✅ Sharp band",IF($J$10&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.6% (fair +102). Your call.</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="16">
+        <f>IF(OR($H$10="",$O$10=""),"",(1+IF($H$10&lt;0,-100/$H$10,$H$10/100))/(1+IF($O$10&lt;0,-100/$O$10,$O$10/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>0.5459000000000001</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>-115</v>
+      </c>
+      <c r="I11" s="13">
+        <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>IF($H$11="","",$F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>IF($H$11="","",MAX(0,($F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))/IF($H$11&lt;0,-100/$H$11,$H$11/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L11" s="18">
+        <f>IF($H$11="","",ROUND(MIN($K$11,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M11" s="12">
+        <f>IF($J$11="","",IF($J$11&lt;0,"Pass",IF($J$11&lt;'Settings'!$B$4,"Thin",IF($J$11&lt;0.06,"✅ Sharp band",IF($J$11&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.6% (fair -120). Your call.</t>
+        </is>
+      </c>
+      <c r="O11" s="15" t="n"/>
+      <c r="P11" s="16">
+        <f>IF(OR($H$11="",$O$11=""),"",(1+IF($H$11&lt;0,-100/$H$11,$H$11/100))/(1+IF($O$11&lt;0,-100/$O$11,$O$11/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J9">
+  <conditionalFormatting sqref="J5:J11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1872,13 +2004,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4736</v>
+        <v>0.4714</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1902,7 +2034,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 47.1% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1938,13 +2070,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5264</v>
+        <v>0.5286</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-111</v>
+        <v>-112</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1968,7 +2100,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -2136,13 +2268,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5518</v>
+        <v>0.545</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-123</v>
+        <v>-120</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2166,7 +2298,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2202,13 +2334,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4482</v>
+        <v>0.455</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>104</v>
+        <v>-103</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2232,7 +2364,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 44.8% (fair +123). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2670,7 +2802,7 @@
         <v>1157</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>614</v>
+        <v>600</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -2796,10 +2928,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4947</v>
+        <v>0.5043</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>102</v>
+        <v>-102</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>100</v>
@@ -2826,7 +2958,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2862,13 +2994,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5053000000000001</v>
+        <v>0.4957</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-108</v>
+        <v>108</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -2892,7 +3024,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2928,13 +3060,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4895</v>
+        <v>0.492</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -2958,7 +3090,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +104). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -2994,13 +3126,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5105</v>
+        <v>0.508</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-104</v>
+        <v>-103</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -3024,7 +3156,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -4973,7 +5105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q104"/>
+  <dimension ref="A1:Q107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4990,340 +5122,127 @@
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="29" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>Washington Mystics offense vs Toronto Tempo defense</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="30" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B75" s="30" t="inlineStr">
+      <c r="B78" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C75" s="30" t="inlineStr">
+      <c r="C78" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D75" s="30" t="inlineStr">
+      <c r="D78" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E75" s="30" t="inlineStr">
+      <c r="E78" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F75" s="30" t="inlineStr">
+      <c r="F78" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G75" s="30" t="inlineStr">
+      <c r="G78" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H75" s="30" t="inlineStr">
+      <c r="H78" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I75" s="30" t="inlineStr">
+      <c r="I78" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J75" s="30" t="inlineStr">
+      <c r="J78" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K75" s="30" t="inlineStr">
+      <c r="K78" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L75" s="30" t="inlineStr">
+      <c r="L78" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M75" s="30" t="inlineStr">
+      <c r="M78" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N75" s="30" t="inlineStr">
+      <c r="N78" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O75" s="30" t="inlineStr">
+      <c r="O78" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P75" s="30" t="inlineStr">
+      <c r="P78" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q75" s="30" t="inlineStr">
+      <c r="Q78" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B76" s="32" t="n">
-        <v>84.111</v>
-      </c>
-      <c r="C76" s="32" t="n">
-        <v>77.967</v>
-      </c>
-      <c r="D76" s="32" t="n">
-        <v>77.15000000000001</v>
-      </c>
-      <c r="E76" s="32" t="n">
-        <v>77.333</v>
-      </c>
-      <c r="F76" s="32" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="G76" s="32" t="n">
-        <v>81.8</v>
-      </c>
-      <c r="H76" s="34" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="I76" s="32" t="inlineStr"/>
-      <c r="J76" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q76" s="33" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B77" s="32" t="n">
-        <v>102.123</v>
-      </c>
-      <c r="C77" s="32" t="n">
-        <v>98.505</v>
-      </c>
-      <c r="D77" s="32" t="n">
-        <v>97.01300000000001</v>
-      </c>
-      <c r="E77" s="32" t="n">
-        <v>96.20099999999999</v>
-      </c>
-      <c r="F77" s="32" t="n">
-        <v>100.864</v>
-      </c>
-      <c r="G77" s="32" t="n">
-        <v>103.268</v>
-      </c>
-      <c r="H77" s="34" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="I77" s="32" t="inlineStr"/>
-      <c r="J77" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q77" s="33" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B78" s="32" t="n">
-        <v>0.501</v>
-      </c>
-      <c r="C78" s="32" t="n">
-        <v>0.496</v>
-      </c>
-      <c r="D78" s="32" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="E78" s="32" t="n">
-        <v>0.479</v>
-      </c>
-      <c r="F78" s="32" t="n">
-        <v>0.498</v>
-      </c>
-      <c r="G78" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="H78" s="34" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="I78" s="32" t="inlineStr"/>
-      <c r="J78" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q78" s="33" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>0.534</v>
+        <v>84.111</v>
       </c>
       <c r="C79" s="32" t="n">
-        <v>0.507</v>
+        <v>77.967</v>
       </c>
       <c r="D79" s="32" t="n">
-        <v>0.504</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="E79" s="32" t="n">
-        <v>0.504</v>
+        <v>77.333</v>
       </c>
       <c r="F79" s="32" t="n">
-        <v>0.529</v>
+        <v>82.3</v>
       </c>
       <c r="G79" s="32" t="n">
-        <v>0.525</v>
+        <v>81.8</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>8th</t>
         </is>
       </c>
       <c r="I79" s="32" t="inlineStr"/>
@@ -5364,37 +5283,37 @@
       </c>
       <c r="Q79" s="33" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>0.296</v>
+        <v>102.123</v>
       </c>
       <c r="C80" s="32" t="n">
-        <v>0.316</v>
+        <v>98.505</v>
       </c>
       <c r="D80" s="32" t="n">
-        <v>0.311</v>
+        <v>97.01300000000001</v>
       </c>
       <c r="E80" s="32" t="n">
-        <v>0.29</v>
+        <v>96.20099999999999</v>
       </c>
       <c r="F80" s="32" t="n">
-        <v>0.298</v>
+        <v>100.864</v>
       </c>
       <c r="G80" s="32" t="n">
-        <v>0.306</v>
+        <v>103.268</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
-          <t>9th</t>
+          <t>8th</t>
         </is>
       </c>
       <c r="I80" s="32" t="inlineStr"/>
@@ -5435,37 +5354,37 @@
       </c>
       <c r="Q80" s="33" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>0.74</v>
+        <v>0.501</v>
       </c>
       <c r="C81" s="32" t="n">
-        <v>0.754</v>
+        <v>0.496</v>
       </c>
       <c r="D81" s="32" t="n">
-        <v>0.738</v>
+        <v>0.488</v>
       </c>
       <c r="E81" s="32" t="n">
-        <v>0.72</v>
+        <v>0.479</v>
       </c>
       <c r="F81" s="32" t="n">
-        <v>0.72</v>
+        <v>0.498</v>
       </c>
       <c r="G81" s="32" t="n">
-        <v>0.781</v>
+        <v>0.497</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
-          <t>8th</t>
+          <t>9th</t>
         </is>
       </c>
       <c r="I81" s="32" t="inlineStr"/>
@@ -5506,37 +5425,37 @@
       </c>
       <c r="Q81" s="33" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B82" s="32" t="n">
-        <v>82.21299999999999</v>
+        <v>0.534</v>
       </c>
       <c r="C82" s="32" t="n">
-        <v>79.015</v>
+        <v>0.507</v>
       </c>
       <c r="D82" s="32" t="n">
-        <v>79.324</v>
+        <v>0.504</v>
       </c>
       <c r="E82" s="32" t="n">
-        <v>80.083</v>
+        <v>0.504</v>
       </c>
       <c r="F82" s="32" t="n">
-        <v>81.364</v>
+        <v>0.529</v>
       </c>
       <c r="G82" s="32" t="n">
-        <v>79.14400000000001</v>
-      </c>
-      <c r="H82" s="35" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.525</v>
+      </c>
+      <c r="H82" s="34" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I82" s="32" t="inlineStr"/>
@@ -5577,37 +5496,37 @@
       </c>
       <c r="Q82" s="33" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>0.554</v>
+        <v>0.296</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>0.54</v>
+        <v>0.316</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>0.532</v>
+        <v>0.311</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>0.521</v>
+        <v>0.29</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>0.547</v>
+        <v>0.298</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.306</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
-          <t>6th</t>
+          <t>9th</t>
         </is>
       </c>
       <c r="I83" s="32" t="inlineStr"/>
@@ -5648,37 +5567,37 @@
       </c>
       <c r="Q83" s="33" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.291</v>
+        <v>0.74</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.233</v>
+        <v>0.754</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.23</v>
+        <v>0.738</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.239</v>
+        <v>0.72</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.266</v>
+        <v>0.72</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.279</v>
-      </c>
-      <c r="H84" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
+        <v>0.781</v>
+      </c>
+      <c r="H84" s="34" t="inlineStr">
+        <is>
+          <t>8th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
@@ -5719,37 +5638,37 @@
       </c>
       <c r="Q84" s="33" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>35.889</v>
+        <v>82.21299999999999</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>32.3</v>
+        <v>79.015</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>33.3</v>
+        <v>79.324</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>33.533</v>
+        <v>80.083</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>35.2</v>
+        <v>81.364</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="H85" s="34" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>79.14400000000001</v>
+      </c>
+      <c r="H85" s="35" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
@@ -5790,37 +5709,37 @@
       </c>
       <c r="Q85" s="33" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>18.778</v>
+        <v>0.554</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>19.733</v>
+        <v>0.54</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>19.45</v>
+        <v>0.532</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>19</v>
+        <v>0.521</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>19.3</v>
+        <v>0.547</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="H86" s="35" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="H86" s="34" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
@@ -5861,37 +5780,37 @@
       </c>
       <c r="Q86" s="33" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>10.778</v>
+        <v>0.291</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>10.3</v>
+        <v>0.233</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>9.800000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>10.067</v>
+        <v>0.239</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>10.5</v>
+        <v>0.266</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="H87" s="35" t="inlineStr">
-        <is>
-          <t>14th</t>
+        <v>0.279</v>
+      </c>
+      <c r="H87" s="36" t="inlineStr">
+        <is>
+          <t>3rd</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
@@ -5932,37 +5851,37 @@
       </c>
       <c r="Q87" s="33" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>15.667</v>
+        <v>35.889</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>14.167</v>
+        <v>32.3</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>14.3</v>
+        <v>33.3</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>14.067</v>
+        <v>33.533</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>14.9</v>
+        <v>35.2</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>14.8</v>
+        <v>33.4</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
-          <t>8th</t>
+          <t>7th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
@@ -6003,321 +5922,321 @@
       </c>
       <c r="Q88" s="33" t="inlineStr">
         <is>
+          <t>Opp REB</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B89" s="32" t="n">
+        <v>18.778</v>
+      </c>
+      <c r="C89" s="32" t="n">
+        <v>19.733</v>
+      </c>
+      <c r="D89" s="32" t="n">
+        <v>19.45</v>
+      </c>
+      <c r="E89" s="32" t="n">
+        <v>19</v>
+      </c>
+      <c r="F89" s="32" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G89" s="32" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="H89" s="35" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I89" s="32" t="inlineStr"/>
+      <c r="J89" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K89" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L89" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M89" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N89" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O89" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P89" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q89" s="33" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B90" s="32" t="n">
+        <v>10.778</v>
+      </c>
+      <c r="C90" s="32" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D90" s="32" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E90" s="32" t="n">
+        <v>10.067</v>
+      </c>
+      <c r="F90" s="32" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G90" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="H90" s="35" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="I90" s="32" t="inlineStr"/>
+      <c r="J90" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q90" s="33" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="31" t="inlineStr">
+        <is>
+          <t>TOV</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="n">
+        <v>15.667</v>
+      </c>
+      <c r="C91" s="32" t="n">
+        <v>14.167</v>
+      </c>
+      <c r="D91" s="32" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="E91" s="32" t="n">
+        <v>14.067</v>
+      </c>
+      <c r="F91" s="32" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G91" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H91" s="34" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="I91" s="32" t="inlineStr"/>
+      <c r="J91" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K91" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L91" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M91" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N91" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O91" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P91" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q91" s="33" t="inlineStr">
+        <is>
           <t>Opp TOV</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="29" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="29" t="inlineStr">
         <is>
           <t>Toronto Tempo offense vs Washington Mystics defense</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="30" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B91" s="30" t="inlineStr">
+      <c r="B94" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C91" s="30" t="inlineStr">
+      <c r="C94" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D91" s="30" t="inlineStr">
+      <c r="D94" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E91" s="30" t="inlineStr">
+      <c r="E94" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F91" s="30" t="inlineStr">
+      <c r="F94" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G91" s="30" t="inlineStr">
+      <c r="G94" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H91" s="30" t="inlineStr">
+      <c r="H94" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I91" s="30" t="inlineStr">
+      <c r="I94" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J91" s="30" t="inlineStr">
+      <c r="J94" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K91" s="30" t="inlineStr">
+      <c r="K94" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L91" s="30" t="inlineStr">
+      <c r="L94" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M91" s="30" t="inlineStr">
+      <c r="M94" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N91" s="30" t="inlineStr">
+      <c r="N94" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O91" s="30" t="inlineStr">
+      <c r="O94" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P91" s="30" t="inlineStr">
+      <c r="P94" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q91" s="30" t="inlineStr">
+      <c r="Q94" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H92" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I92" s="32" t="inlineStr"/>
-      <c r="J92" s="34" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="K92" s="32" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="L92" s="32" t="n">
-        <v>84.889</v>
-      </c>
-      <c r="M92" s="32" t="n">
-        <v>85.857</v>
-      </c>
-      <c r="N92" s="32" t="n">
-        <v>84.73699999999999</v>
-      </c>
-      <c r="O92" s="32" t="n">
-        <v>83.345</v>
-      </c>
-      <c r="P92" s="32" t="n">
-        <v>86.125</v>
-      </c>
-      <c r="Q92" s="33" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I93" s="32" t="inlineStr"/>
-      <c r="J93" s="35" t="inlineStr">
-        <is>
-          <t>13th</t>
-        </is>
-      </c>
-      <c r="K93" s="32" t="n">
-        <v>104.949</v>
-      </c>
-      <c r="L93" s="32" t="n">
-        <v>102.664</v>
-      </c>
-      <c r="M93" s="32" t="n">
-        <v>107.012</v>
-      </c>
-      <c r="N93" s="32" t="n">
-        <v>106.29</v>
-      </c>
-      <c r="O93" s="32" t="n">
-        <v>105.092</v>
-      </c>
-      <c r="P93" s="32" t="n">
-        <v>103.328</v>
-      </c>
-      <c r="Q93" s="33" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H94" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I94" s="32" t="inlineStr"/>
-      <c r="J94" s="35" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="K94" s="32" t="n">
-        <v>0.504</v>
-      </c>
-      <c r="L94" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="M94" s="32" t="n">
-        <v>0.518</v>
-      </c>
-      <c r="N94" s="32" t="n">
-        <v>0.516</v>
-      </c>
-      <c r="O94" s="32" t="n">
-        <v>0.519</v>
-      </c>
-      <c r="P94" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="Q94" s="33" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B95" s="32" t="inlineStr">
@@ -6358,37 +6277,37 @@
       <c r="I95" s="32" t="inlineStr"/>
       <c r="J95" s="34" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>8th</t>
         </is>
       </c>
       <c r="K95" s="32" t="n">
-        <v>0.474</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="L95" s="32" t="n">
-        <v>0.484</v>
+        <v>84.889</v>
       </c>
       <c r="M95" s="32" t="n">
-        <v>0.508</v>
+        <v>85.857</v>
       </c>
       <c r="N95" s="32" t="n">
-        <v>0.508</v>
+        <v>84.73699999999999</v>
       </c>
       <c r="O95" s="32" t="n">
-        <v>0.512</v>
+        <v>83.345</v>
       </c>
       <c r="P95" s="32" t="n">
-        <v>0.484</v>
+        <v>86.125</v>
       </c>
       <c r="Q95" s="33" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B96" s="32" t="inlineStr">
@@ -6429,37 +6348,37 @@
       <c r="I96" s="32" t="inlineStr"/>
       <c r="J96" s="35" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>13th</t>
         </is>
       </c>
       <c r="K96" s="32" t="n">
-        <v>0.363</v>
+        <v>104.949</v>
       </c>
       <c r="L96" s="32" t="n">
-        <v>0.338</v>
+        <v>102.664</v>
       </c>
       <c r="M96" s="32" t="n">
-        <v>0.36</v>
+        <v>107.012</v>
       </c>
       <c r="N96" s="32" t="n">
-        <v>0.352</v>
+        <v>106.29</v>
       </c>
       <c r="O96" s="32" t="n">
-        <v>0.347</v>
+        <v>105.092</v>
       </c>
       <c r="P96" s="32" t="n">
-        <v>0.345</v>
+        <v>103.328</v>
       </c>
       <c r="Q96" s="33" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B97" s="32" t="inlineStr">
@@ -6498,51 +6417,39 @@
         </is>
       </c>
       <c r="I97" s="32" t="inlineStr"/>
-      <c r="J97" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K97" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L97" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M97" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N97" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O97" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P97" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J97" s="35" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="K97" s="32" t="n">
+        <v>0.504</v>
+      </c>
+      <c r="L97" s="32" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="M97" s="32" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="N97" s="32" t="n">
+        <v>0.516</v>
+      </c>
+      <c r="O97" s="32" t="n">
+        <v>0.519</v>
+      </c>
+      <c r="P97" s="32" t="n">
+        <v>0.497</v>
       </c>
       <c r="Q97" s="33" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B98" s="32" t="inlineStr">
@@ -6581,51 +6488,39 @@
         </is>
       </c>
       <c r="I98" s="32" t="inlineStr"/>
-      <c r="J98" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K98" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L98" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M98" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N98" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O98" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P98" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J98" s="34" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K98" s="32" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="L98" s="32" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="M98" s="32" t="n">
+        <v>0.508</v>
+      </c>
+      <c r="N98" s="32" t="n">
+        <v>0.508</v>
+      </c>
+      <c r="O98" s="32" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="P98" s="32" t="n">
+        <v>0.484</v>
       </c>
       <c r="Q98" s="33" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B99" s="32" t="inlineStr">
@@ -6664,51 +6559,39 @@
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr"/>
-      <c r="J99" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K99" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L99" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M99" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N99" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O99" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P99" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J99" s="35" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="K99" s="32" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="L99" s="32" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="M99" s="32" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="N99" s="32" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="O99" s="32" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="P99" s="32" t="n">
+        <v>0.345</v>
       </c>
       <c r="Q99" s="33" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B100" s="32" t="inlineStr">
@@ -6784,14 +6667,14 @@
       </c>
       <c r="Q100" s="33" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B101" s="32" t="inlineStr">
@@ -6830,39 +6713,51 @@
         </is>
       </c>
       <c r="I101" s="32" t="inlineStr"/>
-      <c r="J101" s="36" t="inlineStr">
-        <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="L101" s="32" t="n">
-        <v>30.889</v>
-      </c>
-      <c r="M101" s="32" t="n">
-        <v>32.357</v>
-      </c>
-      <c r="N101" s="32" t="n">
-        <v>31.842</v>
-      </c>
-      <c r="O101" s="32" t="n">
-        <v>31.345</v>
-      </c>
-      <c r="P101" s="32" t="n">
-        <v>30.25</v>
+      <c r="J101" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q101" s="33" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B102" s="32" t="inlineStr">
@@ -6938,14 +6833,14 @@
       </c>
       <c r="Q102" s="33" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B103" s="32" t="inlineStr">
@@ -7021,88 +6916,325 @@
       </c>
       <c r="Q103" s="33" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="inlineStr"/>
+      <c r="J104" s="36" t="inlineStr">
+        <is>
+          <t>4th</t>
+        </is>
+      </c>
+      <c r="K104" s="32" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="L104" s="32" t="n">
+        <v>30.889</v>
+      </c>
+      <c r="M104" s="32" t="n">
+        <v>32.357</v>
+      </c>
+      <c r="N104" s="32" t="n">
+        <v>31.842</v>
+      </c>
+      <c r="O104" s="32" t="n">
+        <v>31.345</v>
+      </c>
+      <c r="P104" s="32" t="n">
+        <v>30.25</v>
+      </c>
+      <c r="Q104" s="33" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I105" s="32" t="inlineStr"/>
+      <c r="J105" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P105" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q105" s="33" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H106" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I106" s="32" t="inlineStr"/>
+      <c r="J106" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q106" s="33" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="31" t="inlineStr">
+        <is>
           <t>TOV</t>
         </is>
       </c>
-      <c r="B104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H104" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I104" s="32" t="inlineStr"/>
-      <c r="J104" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q104" s="33" t="inlineStr">
+      <c r="B107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H107" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I107" s="32" t="inlineStr"/>
+      <c r="J107" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P107" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q107" s="33" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 21:06Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 15:27</t>
+          <t>2026-07-14 17:06</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5286</v>
+        <v>0.533</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-112</v>
+        <v>-114</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1174,17 +1174,17 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -1194,14 +1194,14 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo +1.5</t>
+          <t>Los Angeles Sparks +12.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.545</v>
+        <v>0.5105</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-120</v>
+        <v>-104</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>104</v>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1240,17 +1240,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Golden State Valkyries @ Indiana Fever</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1260,17 +1260,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 168.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5165</v>
+        <v>0.5417</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-107</v>
+        <v>-118</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>-110</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1303,273 +1303,9 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>Over 168.5</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>0.5395</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <v>-117</v>
-      </c>
-      <c r="H8" s="15" t="n">
-        <v>-106</v>
-      </c>
-      <c r="I8" s="13">
-        <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
-        <v/>
-      </c>
-      <c r="J8" s="16">
-        <f>IF($H$8="","",$F$8*IF($H$8&lt;0,-100/$H$8,$H$8/100)-(1-$F$8))</f>
-        <v/>
-      </c>
-      <c r="K8" s="17">
-        <f>IF($H$8="","",MAX(0,($F$8*IF($H$8&lt;0,-100/$H$8,$H$8/100)-(1-$F$8))/IF($H$8&lt;0,-100/$H$8,$H$8/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L8" s="18">
-        <f>IF($H$8="","",ROUND(MIN($K$8,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M8" s="12">
-        <f>IF($J$8="","",IF($J$8&lt;0,"Pass",IF($J$8&lt;'Settings'!$B$4,"Thin",IF($J$8&lt;0.06,"✅ Sharp band",IF($J$8&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N8" s="19" t="inlineStr">
-        <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
-        </is>
-      </c>
-      <c r="O8" s="15" t="n"/>
-      <c r="P8" s="16">
-        <f>IF(OR($H$8="",$O$8=""),"",(1+IF($H$8&lt;0,-100/$H$8,$H$8/100))/(1+IF($O$8&lt;0,-100/$O$8,$O$8/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks @ Minnesota Lynx</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks +12.5</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>0.508</v>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>-103</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>104</v>
-      </c>
-      <c r="I9" s="13">
-        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="16">
-        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="17">
-        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L9" s="18">
-        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M9" s="12">
-        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N9" s="19" t="inlineStr">
-        <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
-        </is>
-      </c>
-      <c r="O9" s="15" t="n"/>
-      <c r="P9" s="16">
-        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks @ Minnesota Lynx</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Under 183.5</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>0.4957</v>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>102</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <v>108</v>
-      </c>
-      <c r="I10" s="13">
-        <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
-        <v/>
-      </c>
-      <c r="J10" s="16">
-        <f>IF($H$10="","",$F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="17">
-        <f>IF($H$10="","",MAX(0,($F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))/IF($H$10&lt;0,-100/$H$10,$H$10/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L10" s="18">
-        <f>IF($H$10="","",ROUND(MIN($K$10,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M10" s="12">
-        <f>IF($J$10="","",IF($J$10&lt;0,"Pass",IF($J$10&lt;'Settings'!$B$4,"Thin",IF($J$10&lt;0.06,"✅ Sharp band",IF($J$10&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N10" s="19" t="inlineStr">
-        <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
-        </is>
-      </c>
-      <c r="O10" s="15" t="n"/>
-      <c r="P10" s="16">
-        <f>IF(OR($H$10="",$O$10=""),"",(1+IF($H$10&lt;0,-100/$H$10,$H$10/100))/(1+IF($O$10&lt;0,-100/$O$10,$O$10/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Indiana Fever</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="n">
-        <v>0.5459000000000001</v>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>-120</v>
-      </c>
-      <c r="H11" s="15" t="n">
-        <v>-115</v>
-      </c>
-      <c r="I11" s="13">
-        <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
-        <v/>
-      </c>
-      <c r="J11" s="16">
-        <f>IF($H$11="","",$F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="17">
-        <f>IF($H$11="","",MAX(0,($F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))/IF($H$11&lt;0,-100/$H$11,$H$11/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L11" s="18">
-        <f>IF($H$11="","",ROUND(MIN($K$11,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M11" s="12">
-        <f>IF($J$11="","",IF($J$11&lt;0,"Pass",IF($J$11&lt;'Settings'!$B$4,"Thin",IF($J$11&lt;0.06,"✅ Sharp band",IF($J$11&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N11" s="19" t="inlineStr">
-        <is>
-          <t>Model 54.6% (fair -120). Your call.</t>
-        </is>
-      </c>
-      <c r="O11" s="15" t="n"/>
-      <c r="P11" s="16">
-        <f>IF(OR($H$11="",$O$11=""),"",(1+IF($H$11&lt;0,-100/$H$11,$H$11/100))/(1+IF($O$11&lt;0,-100/$O$11,$O$11/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J11">
+  <conditionalFormatting sqref="J5:J7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -2004,13 +1740,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4714</v>
+        <v>0.467</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-113</v>
+        <v>-108</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -2034,7 +1770,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -2070,13 +1806,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5286</v>
+        <v>0.533</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-112</v>
+        <v>-114</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -2100,7 +1836,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -2136,10 +1872,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5165</v>
+        <v>0.5428621668460131</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-107</v>
+        <v>-119</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>108</v>
@@ -2166,7 +1902,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2202,13 +1938,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4835</v>
+        <v>0.4571378331539869</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2232,7 +1968,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2268,10 +2004,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.545</v>
+        <v>0.5985540866528527</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-120</v>
+        <v>-149</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>104</v>
@@ -2298,7 +2034,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 59.9% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2334,13 +2070,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.455</v>
+        <v>0.4014459133471473</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-103</v>
+        <v>105</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2364,7 +2100,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 45.5% (fair +120). Your call.</t>
+          <t>Model 40.1% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2928,13 +2664,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5043</v>
+        <v>0.4969</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-102</v>
+        <v>101</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -2958,7 +2694,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2994,13 +2730,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4957</v>
+        <v>0.5031</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>102</v>
+        <v>-101</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -3024,7 +2760,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -3060,13 +2796,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.492</v>
+        <v>0.4895</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -3090,7 +2826,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 48.9% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -3126,10 +2862,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.508</v>
+        <v>0.5105</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-103</v>
+        <v>-104</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>104</v>
@@ -3156,7 +2892,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -3192,13 +2928,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4540999999999999</v>
+        <v>0.445452</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -3222,7 +2958,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.4% (fair +120). Your call.</t>
+          <t>Model 44.5% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -3258,10 +2994,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.554548</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-120</v>
+        <v>-124</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>-115</v>
@@ -3288,7 +3024,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 54.6% (fair -120). Your call.</t>
+          <t>Model 55.5% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -3324,13 +3060,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5395</v>
+        <v>0.5417</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-117</v>
+        <v>-118</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-106</v>
+        <v>-110</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3354,7 +3090,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3390,10 +3126,10 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4605</v>
+        <v>0.4583</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>108</v>
@@ -3420,7 +3156,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 23:02Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 17:06</t>
+          <t>2026-07-14 19:02</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.533</v>
+        <v>0.5301</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-114</v>
+        <v>-113</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1179,32 +1179,32 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Minnesota Lynx</t>
+          <t>Golden State Valkyries @ Indiana Fever</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks +12.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5105</v>
+        <v>0.5497</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-104</v>
+        <v>-122</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>104</v>
+        <v>-108</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1237,75 +1237,9 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Over 168.5</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>0.5417</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>-118</v>
-      </c>
-      <c r="H7" s="15" t="n">
-        <v>-110</v>
-      </c>
-      <c r="I7" s="13">
-        <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
-        <v/>
-      </c>
-      <c r="J7" s="16">
-        <f>IF($H$7="","",$F$7*IF($H$7&lt;0,-100/$H$7,$H$7/100)-(1-$F$7))</f>
-        <v/>
-      </c>
-      <c r="K7" s="17">
-        <f>IF($H$7="","",MAX(0,($F$7*IF($H$7&lt;0,-100/$H$7,$H$7/100)-(1-$F$7))/IF($H$7&lt;0,-100/$H$7,$H$7/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L7" s="18">
-        <f>IF($H$7="","",ROUND(MIN($K$7,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M7" s="12">
-        <f>IF($J$7="","",IF($J$7&lt;0,"Pass",IF($J$7&lt;'Settings'!$B$4,"Thin",IF($J$7&lt;0.06,"✅ Sharp band",IF($J$7&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N7" s="19" t="inlineStr">
-        <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
-        </is>
-      </c>
-      <c r="O7" s="15" t="n"/>
-      <c r="P7" s="16">
-        <f>IF(OR($H$7="",$O$7=""),"",(1+IF($H$7&lt;0,-100/$H$7,$H$7/100))/(1+IF($O$7&lt;0,-100/$O$7,$O$7/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J7">
+  <conditionalFormatting sqref="J5:J6">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1740,13 +1674,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.467</v>
+        <v>0.4699</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1770,7 +1704,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1806,13 +1740,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.533</v>
+        <v>0.5301</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-114</v>
+        <v>-113</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1836,7 +1770,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1868,17 +1802,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 172</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5428621668460131</v>
+        <v>0.5776488749976683</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-119</v>
+        <v>-137</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1902,7 +1836,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1934,17 +1868,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 173.5</t>
+          <t>Under 172</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4571378331539869</v>
+        <v>0.3993511250023317</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>119</v>
+        <v>150</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1968,7 +1902,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 39.9% (fair +150). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2010,7 +1944,7 @@
         <v>-149</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2076,7 +2010,7 @@
         <v>149</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2142,7 +2076,7 @@
         <v>146</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -2208,7 +2142,7 @@
         <v>-146</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -2274,7 +2208,7 @@
         <v>-146</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2396,17 +2330,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky -3.5</t>
+          <t>Chicago Sky -2.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.495</v>
+        <v>0.5166439410560739</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>102</v>
+        <v>-107</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2430,7 +2364,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -2462,17 +2396,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm +3.5</t>
+          <t>Seattle Storm +2.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.505</v>
+        <v>0.4833560589439261</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-102</v>
+        <v>107</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2496,7 +2430,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 48.3% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -2538,7 +2472,7 @@
         <v>1157</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>600</v>
+        <v>575</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -2660,14 +2594,14 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Over 182.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4969</v>
+        <v>0.5222822354138622</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>101</v>
+        <v>-109</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>104</v>
@@ -2694,7 +2628,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2726,17 +2660,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 183.5</t>
+          <t>Under 182.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5031</v>
+        <v>0.4777177645861378</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-101</v>
+        <v>109</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -2760,7 +2694,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2796,10 +2730,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4895</v>
+        <v>0.484</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>104</v>
@@ -2826,7 +2760,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +104). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -2862,13 +2796,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5105</v>
+        <v>0.516</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-104</v>
+        <v>-107</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>104</v>
+        <v>-105</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -2892,7 +2826,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -3056,17 +2990,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5417</v>
+        <v>0.5497</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-118</v>
+        <v>-122</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3090,7 +3024,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3122,17 +3056,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 168.5</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4583</v>
+        <v>0.4503</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -3156,7 +3090,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -3188,17 +3122,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -1.5</t>
+          <t>Indiana Fever -3.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5003</v>
+        <v>0.4284526556424175</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-100</v>
+        <v>133</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -3222,7 +3156,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair -100). Your call.</t>
+          <t>Model 42.8% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -3254,17 +3188,17 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries +1.5</t>
+          <t>Golden State Valkyries +3.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4997</v>
+        <v>0.5715473443575825</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>100</v>
+        <v>-133</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -3288,7 +3222,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair +100). Your call.</t>
+          <t>Model 57.2% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-15 00:05Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-14.xlsx
+++ b/data/output/workbook/2026-07-14.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14 19:02</t>
+          <t>2026-07-14 20:04</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1174,37 +1174,37 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Toronto Tempo +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5497</v>
+        <v>0.5505</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-122</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1237,9 +1237,75 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Over 169.5</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>0.5248</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="I7" s="13">
+        <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
+        <v/>
+      </c>
+      <c r="J7" s="16">
+        <f>IF($H$7="","",$F$7*IF($H$7&lt;0,-100/$H$7,$H$7/100)-(1-$F$7))</f>
+        <v/>
+      </c>
+      <c r="K7" s="17">
+        <f>IF($H$7="","",MAX(0,($F$7*IF($H$7&lt;0,-100/$H$7,$H$7/100)-(1-$F$7))/IF($H$7&lt;0,-100/$H$7,$H$7/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L7" s="18">
+        <f>IF($H$7="","",ROUND(MIN($K$7,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M7" s="12">
+        <f>IF($J$7="","",IF($J$7&lt;0,"Pass",IF($J$7&lt;'Settings'!$B$4,"Thin",IF($J$7&lt;0.06,"✅ Sharp band",IF($J$7&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>Model 52.5% (fair -110). Your call.</t>
+        </is>
+      </c>
+      <c r="O7" s="15" t="n"/>
+      <c r="P7" s="16">
+        <f>IF(OR($H$7="",$O$7=""),"",(1+IF($H$7&lt;0,-100/$H$7,$H$7/100))/(1+IF($O$7&lt;0,-100/$O$7,$O$7/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J6">
+  <conditionalFormatting sqref="J5:J7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1802,17 +1868,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 172</t>
+          <t>Over 172.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5776488749976683</v>
+        <v>0.5661066863084717</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-137</v>
+        <v>-130</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1836,7 +1902,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 56.6% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1868,14 +1934,14 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 172</t>
+          <t>Under 172.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3993511250023317</v>
+        <v>0.4338933136915283</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>108</v>
@@ -1902,7 +1968,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +150). Your call.</t>
+          <t>Model 43.4% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1938,13 +2004,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5985540866528527</v>
+        <v>0.5505</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-149</v>
+        <v>-122</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1968,7 +2034,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 59.9% (fair -149). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2004,13 +2070,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4014459133471473</v>
+        <v>0.4495</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>149</v>
+        <v>122</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2034,7 +2100,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +149). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2198,17 +2264,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 172.5</t>
+          <t>Over 171.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5941506978584125</v>
+        <v>0.6167891999123074</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-146</v>
+        <v>-161</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2232,7 +2298,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 59.4% (fair -146). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2264,17 +2330,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 172.5</t>
+          <t>Under 171.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4058493021415875</v>
+        <v>0.3832108000876926</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -2298,7 +2364,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 40.6% (fair +146). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2330,17 +2396,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky -2.5</t>
+          <t>Chicago Sky -3.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5166439410560739</v>
+        <v>0.4852393637430031</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-107</v>
+        <v>106</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2364,7 +2430,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -2396,14 +2462,14 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm +2.5</t>
+          <t>Seattle Storm +3.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4833560589439261</v>
+        <v>0.5147606362569969</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>107</v>
+        <v>-106</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>104</v>
@@ -2430,7 +2496,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -2594,14 +2660,14 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 182.5</t>
+          <t>Over 183.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5222822354138622</v>
+        <v>0.4939</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-109</v>
+        <v>102</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>104</v>
@@ -2628,7 +2694,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 49.4% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2660,17 +2726,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 182.5</t>
+          <t>Under 183.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4777177645861378</v>
+        <v>0.5061</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>109</v>
+        <v>-102</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>115</v>
+        <v>-105</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -2694,7 +2760,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 50.6% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2990,17 +3056,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 169.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5497</v>
+        <v>0.5248</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-122</v>
+        <v>-110</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3024,7 +3090,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 52.5% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3056,14 +3122,14 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 167.5</t>
+          <t>Under 169.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4503</v>
+        <v>0.4752</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>104</v>
@@ -3090,7 +3156,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 45.0% (fair +122). Your call.</t>
+          <t>Model 47.5% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -3198,7 +3264,7 @@
         <v>-133</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>

</xml_diff>